<commit_message>
feat(import): add bulk import for PM checklist templates
Mẫu bảng kiểm là dữ liệu cha + bảng con, trước đây chỉ tạo tay từng
hạng mục trên màn hình. File PHẲNG: mỗi hàng = 1 hạng mục kiểm tra, cột
của mẫu lặp lại; hệ thống gộp theo (danh mục + loại bảo trì) = khoá định
danh của mẫu, nên người nhập liệu không phải khớp khoá bằng tay.

- import_helpers.py: khai child_table/group_key_fields/parent_fields/
  child_fields ⇒ tự vào GROUPED_IMPORT_DOCTYPES; export trải phẳng cùng
  bố cục để round-trip được
- import_data.py: _do_import_grouped() gộp theo KHOÁ đã chuẩn hoá
  (tên→mã, nhãn VI→giá trị lưu) chứ không theo vị trí liền kề; tạo bản
  ghi qua service layer imm08.create_template, trả thêm groups_created
- import_validators.py: kiểm tra 2 tầng — theo hàng (nội dung, cách ghi
  nhận, ngưỡng) và theo nhóm (mẫu đã tồn tại, khai lệch tên/phiên bản)
- template 07_bang_kiem_bao_tri.xlsx + hàng hướng dẫn trong file 00
- test_import_pm_checklist_template.py: nhóm, bỏ qua dòng lỗi, export
</commit_message>
<xml_diff>
--- a/assetcore/public/import_templates/00_huong_dan_import.xlsx
+++ b/assetcore/public/import_templates/00_huong_dan_import.xlsx
@@ -55,7 +55,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -87,6 +87,11 @@
         <fgColor rgb="00EDE7F6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF9C4"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -114,7 +119,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -141,6 +146,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -508,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -835,17 +843,67 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="9" t="inlineStr">
+    <row r="14" ht="50" customHeight="1">
+      <c r="A14" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>07_bang_kiem_bao_tri.xlsx</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Mẫu bảng kiểm bảo trì định kỳ theo danh mục
+(mỗi hàng = 1 hạng mục kiểm tra)</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>4 — Sau Danh mục tài sản</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Gộp theo Danh mục + Loại bảo trì; mỗi danh mục 1 mẫu/loại</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="9" t="inlineStr">
         <is>
           <t>QUY ƯỚC MÀU:  ■ Đỏ đậm = cột bắt buộc   ■ Xanh đậm = cột tùy chọn   ■ Xanh nhạt = hàng mô tả   ■ Xanh lá = hàng ví dụ</t>
         </is>
       </c>
     </row>
+    <row r="17" ht="32" customHeight="1">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>1. Điền dữ liệu từ HÀNG 6 trở xuống. Hàng 1-5 (banner, tên trường, nhãn, mô tả, ví dụ) là phần khung — không xoá, không ghi đè.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="32" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>2. Cột tham chiếu (Danh mục, Khoa/Phòng, Vị trí, Model, Nhà cung cấp) điền TÊN đúng như trong hệ thống — KHÔNG điền mã hệ thống (AC-DEPT-0007, CAT-0001...). File 'Xuất Excel' cũng in ra tên, dùng lại được ngay.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="32" customHeight="1">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>3. Sai/trùng ở vài dòng KHÔNG chặn cả file: màn hình nhập liệu báo rõ sai ở hàng nào, cột nào; chọn 'Bỏ qua dòng lỗi/trùng' để nhập phần hợp lệ rồi tải báo cáo lỗi về sửa các dòng còn lại.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A15:E15"/>
+  <mergeCells count="5">
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="A19:E19"/>
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A18:E18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(import): add a worked example sheet to the checklist template
- generate_templates.py: sheet 'Ví dụ minh hoạ' bày sẵn 2 mẫu × 3 hạng
  mục để người dùng thấy cách điền nhiều mẫu trong CÙNG một file (không
  cần file riêng, các hàng cùng mẫu không cần liền nhau)
- wb.active = 0 — mở file là thấy sheet nhập liệu, không phải sheet ví dụ;
  parser khoá theo tên sheet nên lưu file lúc đang đứng ở sheet ví dụ vẫn
  nhập đúng
- file 00: thêm mục 'SỬA HÀNG LOẠT dữ liệu đã có' (xuất → sửa → nhập lại)
- sinh lại 10 file .xlsx
</commit_message>
<xml_diff>
--- a/assetcore/public/import_templates/00_huong_dan_import.xlsx
+++ b/assetcore/public/import_templates/00_huong_dan_import.xlsx
@@ -516,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -849,7 +849,8 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>07_bang_kiem_bao_tri.xlsx</t>
+          <t>07_bang_kiem_bao_tri.xlsx
+  → sheet 'Ví dụ minh hoạ'</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
@@ -865,7 +866,7 @@
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>Gộp theo Danh mục + Loại bảo trì; mỗi danh mục 1 mẫu/loại</t>
+          <t>NHIỀU mẫu chung 1 file: điền tiếp xuống dưới, đổi Danh mục / Loại bảo trì. Gộp theo Danh mục + Loại bảo trì; mỗi danh mục 1 mẫu/loại. Mẫu đã có: bật 'Cập nhật mẫu đã có' để thay toàn bộ hạng mục</t>
         </is>
       </c>
     </row>
@@ -897,8 +898,16 @@
         </is>
       </c>
     </row>
+    <row r="20" ht="32" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>4. SỬA HÀNG LOẠT dữ liệu đã có: bấm 'Xuất Excel' → sửa trong file → nhập lại, rồi bật «Cập nhật bản ghi đã có» ở bước kiểm tra. Ô để trống giữ nguyên giá trị cũ (không xoá trắng). Bản ghi được nhận dạng theo MÃ nếu có mã, không có thì theo TÊN. Riêng thiết bị: mã tài sản, số serial và trạng thái vòng đời KHÔNG đổi được bằng file — sửa trên màn hình chi tiết để có phê duyệt và lịch sử thay đổi.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
+    <mergeCell ref="A20:E20"/>
     <mergeCell ref="A16:E16"/>
     <mergeCell ref="A19:E19"/>
     <mergeCell ref="A1:E1"/>

</xml_diff>